<commit_message>
Classification Algorithm and metrics added
Classification Algorithm and metrics added
</commit_message>
<xml_diff>
--- a/10. Classification Algorithm/Summary.xlsx
+++ b/10. Classification Algorithm/Summary.xlsx
@@ -4,18 +4,19 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Types-Regression" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
   <si>
     <t xml:space="preserve">Accuracy </t>
   </si>
@@ -330,13 +331,52 @@
   </si>
   <si>
     <t>What is Support in Machine Learning?  (Purchased)</t>
+  </si>
+  <si>
+    <t>Types of Regression Techniques:</t>
+  </si>
+  <si>
+    <t>1. Linear Regression</t>
+  </si>
+  <si>
+    <t>2. Polynomial Regression</t>
+  </si>
+  <si>
+    <t>3. Stepwise Regression</t>
+  </si>
+  <si>
+    <t>4. Decision Tree Regression</t>
+  </si>
+  <si>
+    <t>5. Random Forest Regression</t>
+  </si>
+  <si>
+    <t>6. Support Vector Regression</t>
+  </si>
+  <si>
+    <t>7. Ridge Regression</t>
+  </si>
+  <si>
+    <t>8. Lasso Regression</t>
+  </si>
+  <si>
+    <t>9. ElasticNet Regression</t>
+  </si>
+  <si>
+    <t>10. Bayesian Linear Regression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.geeksforgeeks.org/machine-learning/types-of-regression-techniques/ </t>
+  </si>
+  <si>
+    <t>https://scikit-learn.org/stable/supervised_learning.html </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -348,6 +388,28 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF4C647D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF4C647D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -385,10 +447,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -415,8 +478,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -987,6 +1058,85 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C2:D12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="77.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C2" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C3" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C4" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C5" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C6" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C7" s="13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C8" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C9" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C10" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C11" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C12" s="13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="D3" r:id="rId2" display="https://scikit-learn.org/stable/supervised_learning.html"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C3:H11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>